<commit_message>
Add excel format for the templates
</commit_message>
<xml_diff>
--- a/capstone-defense-scheduler-backend/src/main/resources/templates/Lecturer_Import_Template.xlsx
+++ b/capstone-defense-scheduler-backend/src/main/resources/templates/Lecturer_Import_Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\01-Workspace\University Project\SWD316\BE\capstone-defense-scheduler-backend\src\main\resources\templates\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{540F3759-36D7-45A8-AA60-DF880D997F0A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E8B3C58-6DAF-48AA-91E7-88CE2E6F481F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="25820" windowHeight="15500" xr2:uid="{F0D7D9FA-C678-45FD-8D6C-E942DB18D234}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="23" uniqueCount="23">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
   <si>
     <t>No</t>
   </si>
@@ -75,9 +75,6 @@
     <t>Max Quota</t>
   </si>
   <si>
-    <t>SE</t>
-  </si>
-  <si>
     <t>Competencies</t>
   </si>
   <si>
@@ -91,18 +88,6 @@
   </si>
   <si>
     <t/>
-  </si>
-  <si>
-    <t>Duong Cong Danh</t>
-  </si>
-  <si>
-    <t>danhdc@fpt.edu.vn</t>
-  </si>
-  <si>
-    <t>SE002</t>
-  </si>
-  <si>
-    <t>0967965791</t>
   </si>
 </sst>
 </file>
@@ -247,11 +232,11 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -880,27 +865,27 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:13" ht="64.5" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A1" s="14" t="s">
+      <c r="A1" s="15" t="s">
+        <v>15</v>
+      </c>
+      <c r="B1" s="15"/>
+      <c r="C1" s="15"/>
+      <c r="D1" s="15"/>
+      <c r="E1" s="15"/>
+      <c r="F1" s="2" t="s">
+        <v>14</v>
+      </c>
+      <c r="G1" s="15" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="15"/>
+      <c r="I1" s="15"/>
+      <c r="J1" s="15"/>
+      <c r="K1" s="15"/>
+      <c r="L1" s="15" t="s">
         <v>16</v>
       </c>
-      <c r="B1" s="14"/>
-      <c r="C1" s="14"/>
-      <c r="D1" s="14"/>
-      <c r="E1" s="14"/>
-      <c r="F1" s="2" t="s">
-        <v>15</v>
-      </c>
-      <c r="G1" s="14" t="s">
-        <v>14</v>
-      </c>
-      <c r="H1" s="14"/>
-      <c r="I1" s="14"/>
-      <c r="J1" s="14"/>
-      <c r="K1" s="14"/>
-      <c r="L1" s="14" t="s">
-        <v>17</v>
-      </c>
-      <c r="M1" s="14"/>
+      <c r="M1" s="15"/>
     </row>
     <row r="2" spans="1:13" ht="27.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3" t="s">
@@ -943,46 +928,20 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="29" x14ac:dyDescent="0.35">
-      <c r="A3" s="1">
-        <v>1</v>
-      </c>
-      <c r="B3" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C3" s="15" t="s">
-        <v>20</v>
-      </c>
-      <c r="D3" s="1" t="s">
-        <v>21</v>
-      </c>
-      <c r="E3" s="11" t="s">
-        <v>22</v>
-      </c>
-      <c r="F3" s="1" t="s">
-        <v>13</v>
-      </c>
-      <c r="G3" s="1">
-        <v>1</v>
-      </c>
-      <c r="H3" s="1">
-        <v>2</v>
-      </c>
-      <c r="I3" s="1">
-        <v>3</v>
-      </c>
-      <c r="J3" s="1">
-        <v>4</v>
-      </c>
-      <c r="K3" s="1">
-        <v>5</v>
-      </c>
-      <c r="L3" s="1">
-        <v>1</v>
-      </c>
-      <c r="M3" s="1">
-        <v>7</v>
-      </c>
+    <row r="3" spans="1:13" x14ac:dyDescent="0.35">
+      <c r="A3" s="1"/>
+      <c r="B3" s="1"/>
+      <c r="C3" s="14"/>
+      <c r="D3" s="1"/>
+      <c r="E3" s="11"/>
+      <c r="F3" s="1"/>
+      <c r="G3" s="1"/>
+      <c r="H3" s="1"/>
+      <c r="I3" s="1"/>
+      <c r="J3" s="1"/>
+      <c r="K3" s="1"/>
+      <c r="L3" s="1"/>
+      <c r="M3" s="1"/>
     </row>
     <row r="4" spans="1:13" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
@@ -1018,7 +977,7 @@
       <c r="A6" s="7"/>
       <c r="B6" s="7"/>
       <c r="C6" s="8" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="D6" s="7"/>
       <c r="E6" s="12"/>
@@ -1747,12 +1706,9 @@
       <formula2>11</formula2>
     </dataValidation>
   </dataValidations>
-  <hyperlinks>
-    <hyperlink ref="C3" r:id="rId1" xr:uid="{7E17D00D-F2B4-4C68-97A6-CF56C0485D91}"/>
-  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <tableParts count="1">
-    <tablePart r:id="rId2"/>
+    <tablePart r:id="rId1"/>
   </tableParts>
 </worksheet>
 </file>
</xml_diff>